<commit_message>
Archipelago checks: Spirits tab, 98 spirits scanned from the map files in the ROM
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DOCS/archipelago_checks.xlsx
+++ b/DOCS/archipelago_checks.xlsx
@@ -7,6 +7,7 @@
     <sheet name="Givers" sheetId="3" r:id="rId3"/>
     <sheet name="Enemies" sheetId="4" r:id="rId4"/>
     <sheet name="Bosses" sheetId="5" r:id="rId5"/>
+    <sheet name="Spirits" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -206,303 +207,323 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Spirits</t>
+        </is>
+      </c>
+      <c r="B9" s="0">
+        <v>98</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirits</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every spirit pickup, read from the spirit list at the end of each map file in the ROM: its map, world position and record address. 98 in all, which is also the cap on the game's collected-spirit counter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Total</t>
         </is>
       </c>
-      <c r="B9" s="0">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="B10" s="0">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Suggested location names</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Each sheet has a "Suggested name" column in the form "Category - Place" that is unique across the whole set, so it can be pasted straight into a locations table. Rename freely; the ROM addresses next to them are what a patcher needs.</t>
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Vanilla item pool (ids the tables use)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Id</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Item</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="0">
-        <v>0</v>
-      </c>
-      <c r="B16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Spirit Light</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fresh Bread</t>
+          <t xml:space="preserve">Spirit Light</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Honey Bread</t>
+          <t xml:space="preserve">Fresh Bread</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Healing Potion</t>
+          <t xml:space="preserve">Honey Bread</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dragon's Potion</t>
+          <t xml:space="preserve">Healing Potion</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dew Drop</t>
+          <t xml:space="preserve">Dragon's Potion</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mint Leaves</t>
+          <t xml:space="preserve">Dew Drop</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Heroes Drink</t>
+          <t xml:space="preserve">Mint Leaves</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Silent Flute</t>
+          <t xml:space="preserve">Heroes Drink</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Celine's Bell</t>
+          <t xml:space="preserve">Silent Flute</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Replica</t>
+          <t xml:space="preserve">Celine's Bell</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Giant's Shoes</t>
+          <t xml:space="preserve">Replica</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Silver Amulet</t>
+          <t xml:space="preserve">Giant's Shoes</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Golden Amulet</t>
+          <t xml:space="preserve">Silver Amulet</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">White Wings</t>
+          <t xml:space="preserve">Golden Amulet</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yellow Wings</t>
+          <t xml:space="preserve">White Wings</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blue Wings</t>
+          <t xml:space="preserve">Yellow Wings</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Wings</t>
+          <t xml:space="preserve">Blue Wings</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Red Wings</t>
+          <t xml:space="preserve">Green Wings</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Black Wings</t>
+          <t xml:space="preserve">Red Wings</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Earth Orb</t>
+          <t xml:space="preserve">Black Wings</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wind Jade</t>
+          <t xml:space="preserve">Earth Orb</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water Jewel</t>
+          <t xml:space="preserve">Wind Jade</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fire Ruby</t>
+          <t xml:space="preserve">Water Jewel</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eletale's Book</t>
+          <t xml:space="preserve">Fire Ruby</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0">
+        <v>24</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eletale's Book</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0">
         <v>25</v>
       </c>
-      <c r="B41" s="0" t="inlineStr">
+      <c r="B42" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Dark Gaol Key</t>
         </is>
@@ -10569,4 +10590,3216 @@
   </sheetData>
   <autoFilter ref="A1:M9"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="7" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="9" customWidth="1"/>
+    <col min="7" max="7" width="9" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="70" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Suggested name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Map</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Map #</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nth in map</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Z</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record at</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0">
+        <v>0</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Melrode #1</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Melrode</t>
+        </is>
+      </c>
+      <c r="D2" s="0">
+        <v>0</v>
+      </c>
+      <c r="E2" s="0">
+        <v>1</v>
+      </c>
+      <c r="F2" s="0">
+        <v>-503.5</v>
+      </c>
+      <c r="G2" s="0">
+        <v>0</v>
+      </c>
+      <c r="H2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x135E54</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
+        <v>1</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Melrode #2</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Melrode</t>
+        </is>
+      </c>
+      <c r="D3" s="0">
+        <v>0</v>
+      </c>
+      <c r="E3" s="0">
+        <v>2</v>
+      </c>
+      <c r="F3" s="0">
+        <v>1165</v>
+      </c>
+      <c r="G3" s="0">
+        <v>754.5</v>
+      </c>
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x135E60</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>2</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dondoran #1</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dondoran</t>
+        </is>
+      </c>
+      <c r="D4" s="0">
+        <v>1</v>
+      </c>
+      <c r="E4" s="0">
+        <v>1</v>
+      </c>
+      <c r="F4" s="0">
+        <v>-108</v>
+      </c>
+      <c r="G4" s="0">
+        <v>9</v>
+      </c>
+      <c r="H4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x167F40</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>3</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Holy Plains #1</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Holy Plains</t>
+        </is>
+      </c>
+      <c r="D5" s="0">
+        <v>2</v>
+      </c>
+      <c r="E5" s="0">
+        <v>1</v>
+      </c>
+      <c r="F5" s="0">
+        <v>70</v>
+      </c>
+      <c r="G5" s="0">
+        <v>-982.5</v>
+      </c>
+      <c r="H5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x19E320</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>4</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Holy Plains #2</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Holy Plains</t>
+        </is>
+      </c>
+      <c r="D6" s="0">
+        <v>2</v>
+      </c>
+      <c r="E6" s="0">
+        <v>2</v>
+      </c>
+      <c r="F6" s="0">
+        <v>812.5</v>
+      </c>
+      <c r="G6" s="0">
+        <v>175</v>
+      </c>
+      <c r="H6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x19E32C</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>5</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dondoran Flats #1</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dondoran Flats</t>
+        </is>
+      </c>
+      <c r="D7" s="0">
+        <v>3</v>
+      </c>
+      <c r="E7" s="0">
+        <v>1</v>
+      </c>
+      <c r="F7" s="0">
+        <v>-472.5</v>
+      </c>
+      <c r="G7" s="0">
+        <v>882.5</v>
+      </c>
+      <c r="H7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x1CC9C0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>6</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dondoran Flats #2</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dondoran Flats</t>
+        </is>
+      </c>
+      <c r="D8" s="0">
+        <v>3</v>
+      </c>
+      <c r="E8" s="0">
+        <v>2</v>
+      </c>
+      <c r="F8" s="0">
+        <v>157.5</v>
+      </c>
+      <c r="G8" s="0">
+        <v>7.5</v>
+      </c>
+      <c r="H8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x1CC9CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>7</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dondoran Flats #3</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dondoran Flats</t>
+        </is>
+      </c>
+      <c r="D9" s="0">
+        <v>3</v>
+      </c>
+      <c r="E9" s="0">
+        <v>3</v>
+      </c>
+      <c r="F9" s="0">
+        <v>2.5</v>
+      </c>
+      <c r="G9" s="0">
+        <v>1250</v>
+      </c>
+      <c r="H9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x1CC9D8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>8</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Larapool #1</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Larapool</t>
+        </is>
+      </c>
+      <c r="D10" s="0">
+        <v>4</v>
+      </c>
+      <c r="E10" s="0">
+        <v>1</v>
+      </c>
+      <c r="F10" s="0">
+        <v>243</v>
+      </c>
+      <c r="G10" s="0">
+        <v>-133</v>
+      </c>
+      <c r="H10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x208E20</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>9</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Larapool #2</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Larapool</t>
+        </is>
+      </c>
+      <c r="D11" s="0">
+        <v>4</v>
+      </c>
+      <c r="E11" s="0">
+        <v>2</v>
+      </c>
+      <c r="F11" s="0">
+        <v>16</v>
+      </c>
+      <c r="G11" s="0">
+        <v>366</v>
+      </c>
+      <c r="H11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x208E2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0">
+        <v>10</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Larapool #3</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Larapool</t>
+        </is>
+      </c>
+      <c r="D12" s="0">
+        <v>4</v>
+      </c>
+      <c r="E12" s="0">
+        <v>3</v>
+      </c>
+      <c r="F12" s="0">
+        <v>597</v>
+      </c>
+      <c r="G12" s="0">
+        <v>199</v>
+      </c>
+      <c r="H12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x208E38</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0">
+        <v>11</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - West Carmagh (Greenoch) #1</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Carmagh (Greenoch)</t>
+        </is>
+      </c>
+      <c r="D13" s="0">
+        <v>5</v>
+      </c>
+      <c r="E13" s="0">
+        <v>1</v>
+      </c>
+      <c r="F13" s="0">
+        <v>705</v>
+      </c>
+      <c r="G13" s="0">
+        <v>-55</v>
+      </c>
+      <c r="H13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x253E30</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0">
+        <v>12</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - West Carmagh (Greenoch) #2</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Carmagh (Greenoch)</t>
+        </is>
+      </c>
+      <c r="D14" s="0">
+        <v>5</v>
+      </c>
+      <c r="E14" s="0">
+        <v>2</v>
+      </c>
+      <c r="F14" s="0">
+        <v>55</v>
+      </c>
+      <c r="G14" s="0">
+        <v>515</v>
+      </c>
+      <c r="H14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x253E3C</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0">
+        <v>13</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - West Carmagh (Greenoch) #3</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Carmagh (Greenoch)</t>
+        </is>
+      </c>
+      <c r="D15" s="0">
+        <v>5</v>
+      </c>
+      <c r="E15" s="0">
+        <v>3</v>
+      </c>
+      <c r="F15" s="0">
+        <v>-415</v>
+      </c>
+      <c r="G15" s="0">
+        <v>-650</v>
+      </c>
+      <c r="H15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x253E48</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0">
+        <v>14</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Normoon #1</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Normoon</t>
+        </is>
+      </c>
+      <c r="D16" s="0">
+        <v>6</v>
+      </c>
+      <c r="E16" s="0">
+        <v>1</v>
+      </c>
+      <c r="F16" s="0">
+        <v>200</v>
+      </c>
+      <c r="G16" s="0">
+        <v>152.5</v>
+      </c>
+      <c r="H16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x278960</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0">
+        <v>15</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Normoon #2</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Normoon</t>
+        </is>
+      </c>
+      <c r="D17" s="0">
+        <v>6</v>
+      </c>
+      <c r="E17" s="0">
+        <v>2</v>
+      </c>
+      <c r="F17" s="0">
+        <v>195</v>
+      </c>
+      <c r="G17" s="0">
+        <v>5</v>
+      </c>
+      <c r="H17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x27896C</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0">
+        <v>16</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Normoon #3</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Normoon</t>
+        </is>
+      </c>
+      <c r="D18" s="0">
+        <v>6</v>
+      </c>
+      <c r="E18" s="0">
+        <v>3</v>
+      </c>
+      <c r="F18" s="0">
+        <v>220</v>
+      </c>
+      <c r="G18" s="0">
+        <v>-107.5</v>
+      </c>
+      <c r="H18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x278978</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0">
+        <v>17</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - West Limelin #1</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Limelin</t>
+        </is>
+      </c>
+      <c r="D19" s="0">
+        <v>7</v>
+      </c>
+      <c r="E19" s="0">
+        <v>1</v>
+      </c>
+      <c r="F19" s="0">
+        <v>1105</v>
+      </c>
+      <c r="G19" s="0">
+        <v>-1535</v>
+      </c>
+      <c r="H19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x2AA610</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0">
+        <v>18</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - West Limelin #2</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Limelin</t>
+        </is>
+      </c>
+      <c r="D20" s="0">
+        <v>7</v>
+      </c>
+      <c r="E20" s="0">
+        <v>2</v>
+      </c>
+      <c r="F20" s="0">
+        <v>1180</v>
+      </c>
+      <c r="G20" s="0">
+        <v>-720</v>
+      </c>
+      <c r="H20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x2AA61C</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0">
+        <v>19</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - West Limelin #3</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Limelin</t>
+        </is>
+      </c>
+      <c r="D21" s="0">
+        <v>7</v>
+      </c>
+      <c r="E21" s="0">
+        <v>3</v>
+      </c>
+      <c r="F21" s="0">
+        <v>-800</v>
+      </c>
+      <c r="G21" s="0">
+        <v>-155</v>
+      </c>
+      <c r="H21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x2AA628</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0">
+        <v>20</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - West Limelin #4</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Limelin</t>
+        </is>
+      </c>
+      <c r="D22" s="0">
+        <v>7</v>
+      </c>
+      <c r="E22" s="0">
+        <v>4</v>
+      </c>
+      <c r="F22" s="0">
+        <v>1040</v>
+      </c>
+      <c r="G22" s="0">
+        <v>-1760</v>
+      </c>
+      <c r="H22" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x2AA634</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0">
+        <v>21</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Limelin #1</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limelin</t>
+        </is>
+      </c>
+      <c r="D23" s="0">
+        <v>8</v>
+      </c>
+      <c r="E23" s="0">
+        <v>1</v>
+      </c>
+      <c r="F23" s="0">
+        <v>-768</v>
+      </c>
+      <c r="G23" s="0">
+        <v>462</v>
+      </c>
+      <c r="H23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x2F83F0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0">
+        <v>22</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Limelin #2</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limelin</t>
+        </is>
+      </c>
+      <c r="D24" s="0">
+        <v>8</v>
+      </c>
+      <c r="E24" s="0">
+        <v>2</v>
+      </c>
+      <c r="F24" s="0">
+        <v>-412</v>
+      </c>
+      <c r="G24" s="0">
+        <v>-339</v>
+      </c>
+      <c r="H24" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x2F83FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0">
+        <v>23</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Limelin #3</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limelin</t>
+        </is>
+      </c>
+      <c r="D25" s="0">
+        <v>8</v>
+      </c>
+      <c r="E25" s="0">
+        <v>3</v>
+      </c>
+      <c r="F25" s="0">
+        <v>189</v>
+      </c>
+      <c r="G25" s="0">
+        <v>-405</v>
+      </c>
+      <c r="H25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x2F8408</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0">
+        <v>24</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Limelin #4</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limelin</t>
+        </is>
+      </c>
+      <c r="D26" s="0">
+        <v>8</v>
+      </c>
+      <c r="E26" s="0">
+        <v>4</v>
+      </c>
+      <c r="F26" s="0">
+        <v>670</v>
+      </c>
+      <c r="G26" s="0">
+        <v>239</v>
+      </c>
+      <c r="H26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x2F8414</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0">
+        <v>25</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Limelin #5</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limelin</t>
+        </is>
+      </c>
+      <c r="D27" s="0">
+        <v>8</v>
+      </c>
+      <c r="E27" s="0">
+        <v>5</v>
+      </c>
+      <c r="F27" s="0">
+        <v>0</v>
+      </c>
+      <c r="G27" s="0">
+        <v>170</v>
+      </c>
+      <c r="H27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x2F8420</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0">
+        <v>26</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dindom Dries #1</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dindom Dries</t>
+        </is>
+      </c>
+      <c r="D28" s="0">
+        <v>9</v>
+      </c>
+      <c r="E28" s="0">
+        <v>1</v>
+      </c>
+      <c r="F28" s="0">
+        <v>-1990</v>
+      </c>
+      <c r="G28" s="0">
+        <v>-415</v>
+      </c>
+      <c r="H28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x347910</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0">
+        <v>27</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dindom Dries #2</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dindom Dries</t>
+        </is>
+      </c>
+      <c r="D29" s="0">
+        <v>9</v>
+      </c>
+      <c r="E29" s="0">
+        <v>2</v>
+      </c>
+      <c r="F29" s="0">
+        <v>-1740</v>
+      </c>
+      <c r="G29" s="0">
+        <v>-520</v>
+      </c>
+      <c r="H29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x34791C</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0">
+        <v>28</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dindom Dries #3</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dindom Dries</t>
+        </is>
+      </c>
+      <c r="D30" s="0">
+        <v>9</v>
+      </c>
+      <c r="E30" s="0">
+        <v>3</v>
+      </c>
+      <c r="F30" s="0">
+        <v>325</v>
+      </c>
+      <c r="G30" s="0">
+        <v>-310</v>
+      </c>
+      <c r="H30" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x347928</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0">
+        <v>29</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dindom Dries #4</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dindom Dries</t>
+        </is>
+      </c>
+      <c r="D31" s="0">
+        <v>9</v>
+      </c>
+      <c r="E31" s="0">
+        <v>4</v>
+      </c>
+      <c r="F31" s="0">
+        <v>-680</v>
+      </c>
+      <c r="G31" s="0">
+        <v>350</v>
+      </c>
+      <c r="H31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x347934</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0">
+        <v>30</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dindom Dries #5</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dindom Dries</t>
+        </is>
+      </c>
+      <c r="D32" s="0">
+        <v>9</v>
+      </c>
+      <c r="E32" s="0">
+        <v>5</v>
+      </c>
+      <c r="F32" s="0">
+        <v>2700</v>
+      </c>
+      <c r="G32" s="0">
+        <v>-2100</v>
+      </c>
+      <c r="H32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x347940</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0">
+        <v>31</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dindom Dries #6</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dindom Dries</t>
+        </is>
+      </c>
+      <c r="D33" s="0">
+        <v>9</v>
+      </c>
+      <c r="E33" s="0">
+        <v>6</v>
+      </c>
+      <c r="F33" s="0">
+        <v>-2010</v>
+      </c>
+      <c r="G33" s="0">
+        <v>200</v>
+      </c>
+      <c r="H33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x34794C</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0">
+        <v>32</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Shamwood #1</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shamwood</t>
+        </is>
+      </c>
+      <c r="D34" s="0">
+        <v>10</v>
+      </c>
+      <c r="E34" s="0">
+        <v>1</v>
+      </c>
+      <c r="F34" s="0">
+        <v>-120</v>
+      </c>
+      <c r="G34" s="0">
+        <v>460</v>
+      </c>
+      <c r="H34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x36D930</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0">
+        <v>33</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Shamwood #2</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shamwood</t>
+        </is>
+      </c>
+      <c r="D35" s="0">
+        <v>10</v>
+      </c>
+      <c r="E35" s="0">
+        <v>2</v>
+      </c>
+      <c r="F35" s="0">
+        <v>-82.5</v>
+      </c>
+      <c r="G35" s="0">
+        <v>-1037.5</v>
+      </c>
+      <c r="H35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x36D93C</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0">
+        <v>34</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Shamwood #3</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shamwood</t>
+        </is>
+      </c>
+      <c r="D36" s="0">
+        <v>10</v>
+      </c>
+      <c r="E36" s="0">
+        <v>3</v>
+      </c>
+      <c r="F36" s="0">
+        <v>-115</v>
+      </c>
+      <c r="G36" s="0">
+        <v>122.5</v>
+      </c>
+      <c r="H36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x36D950</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0">
+        <v>35</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Shamwood #4</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shamwood</t>
+        </is>
+      </c>
+      <c r="D37" s="0">
+        <v>10</v>
+      </c>
+      <c r="E37" s="0">
+        <v>4</v>
+      </c>
+      <c r="F37" s="0">
+        <v>30</v>
+      </c>
+      <c r="G37" s="0">
+        <v>225</v>
+      </c>
+      <c r="H37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x36D95C</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0">
+        <v>36</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Brannoch / Baragoon Moor #1</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brannoch / Baragoon Moor</t>
+        </is>
+      </c>
+      <c r="D38" s="0">
+        <v>11</v>
+      </c>
+      <c r="E38" s="0">
+        <v>1</v>
+      </c>
+      <c r="F38" s="0">
+        <v>-2140</v>
+      </c>
+      <c r="G38" s="0">
+        <v>325</v>
+      </c>
+      <c r="H38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x3CB580</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0">
+        <v>37</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Brannoch / Baragoon Moor #2</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brannoch / Baragoon Moor</t>
+        </is>
+      </c>
+      <c r="D39" s="0">
+        <v>11</v>
+      </c>
+      <c r="E39" s="0">
+        <v>2</v>
+      </c>
+      <c r="F39" s="0">
+        <v>484.5</v>
+      </c>
+      <c r="G39" s="0">
+        <v>153</v>
+      </c>
+      <c r="H39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x3CB590</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0">
+        <v>38</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Brannoch / Baragoon Moor #3</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brannoch / Baragoon Moor</t>
+        </is>
+      </c>
+      <c r="D40" s="0">
+        <v>11</v>
+      </c>
+      <c r="E40" s="0">
+        <v>3</v>
+      </c>
+      <c r="F40" s="0">
+        <v>336</v>
+      </c>
+      <c r="G40" s="0">
+        <v>34</v>
+      </c>
+      <c r="H40" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x3CB59C</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0">
+        <v>39</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Brannoch / Baragoon Moor #4</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brannoch / Baragoon Moor</t>
+        </is>
+      </c>
+      <c r="D41" s="0">
+        <v>11</v>
+      </c>
+      <c r="E41" s="0">
+        <v>4</v>
+      </c>
+      <c r="F41" s="0">
+        <v>-586</v>
+      </c>
+      <c r="G41" s="0">
+        <v>220.5</v>
+      </c>
+      <c r="H41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x3CB5A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0">
+        <v>40</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Brannoch / Baragoon Moor #5</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brannoch / Baragoon Moor</t>
+        </is>
+      </c>
+      <c r="D42" s="0">
+        <v>11</v>
+      </c>
+      <c r="E42" s="0">
+        <v>5</v>
+      </c>
+      <c r="F42" s="0">
+        <v>-325</v>
+      </c>
+      <c r="G42" s="0">
+        <v>-324</v>
+      </c>
+      <c r="H42" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x3CB5B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0">
+        <v>41</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Isle of Skye #1</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isle of Skye</t>
+        </is>
+      </c>
+      <c r="D43" s="0">
+        <v>12</v>
+      </c>
+      <c r="E43" s="0">
+        <v>1</v>
+      </c>
+      <c r="F43" s="0">
+        <v>622.5</v>
+      </c>
+      <c r="G43" s="0">
+        <v>-30</v>
+      </c>
+      <c r="H43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x3E3190</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0">
+        <v>42</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Isle of Skye #2</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isle of Skye</t>
+        </is>
+      </c>
+      <c r="D44" s="0">
+        <v>12</v>
+      </c>
+      <c r="E44" s="0">
+        <v>2</v>
+      </c>
+      <c r="F44" s="0">
+        <v>450</v>
+      </c>
+      <c r="G44" s="0">
+        <v>20</v>
+      </c>
+      <c r="H44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x3E319C</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0">
+        <v>43</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Isle of Skye #3</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isle of Skye</t>
+        </is>
+      </c>
+      <c r="D45" s="0">
+        <v>12</v>
+      </c>
+      <c r="E45" s="0">
+        <v>3</v>
+      </c>
+      <c r="F45" s="0">
+        <v>977.5</v>
+      </c>
+      <c r="G45" s="0">
+        <v>465</v>
+      </c>
+      <c r="H45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x3E31A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0">
+        <v>44</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Isle of Skye #4</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isle of Skye</t>
+        </is>
+      </c>
+      <c r="D46" s="0">
+        <v>12</v>
+      </c>
+      <c r="E46" s="0">
+        <v>4</v>
+      </c>
+      <c r="F46" s="0">
+        <v>207.5</v>
+      </c>
+      <c r="G46" s="0">
+        <v>-77.5</v>
+      </c>
+      <c r="H46" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x3E31B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0">
+        <v>45</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Blue Cave #1</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blue Cave</t>
+        </is>
+      </c>
+      <c r="D47" s="0">
+        <v>26</v>
+      </c>
+      <c r="E47" s="0">
+        <v>1</v>
+      </c>
+      <c r="F47" s="0">
+        <v>-800</v>
+      </c>
+      <c r="G47" s="0">
+        <v>1920</v>
+      </c>
+      <c r="H47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x667720</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0">
+        <v>46</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Blue Cave #2</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blue Cave</t>
+        </is>
+      </c>
+      <c r="D48" s="0">
+        <v>26</v>
+      </c>
+      <c r="E48" s="0">
+        <v>2</v>
+      </c>
+      <c r="F48" s="0">
+        <v>-10</v>
+      </c>
+      <c r="G48" s="0">
+        <v>1000</v>
+      </c>
+      <c r="H48" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x66772C</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0">
+        <v>47</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Blue Cave #3</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blue Cave</t>
+        </is>
+      </c>
+      <c r="D49" s="0">
+        <v>26</v>
+      </c>
+      <c r="E49" s="0">
+        <v>3</v>
+      </c>
+      <c r="F49" s="0">
+        <v>1260</v>
+      </c>
+      <c r="G49" s="0">
+        <v>1060</v>
+      </c>
+      <c r="H49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x667738</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0">
+        <v>48</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Blue Cave #4</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blue Cave</t>
+        </is>
+      </c>
+      <c r="D50" s="0">
+        <v>26</v>
+      </c>
+      <c r="E50" s="0">
+        <v>4</v>
+      </c>
+      <c r="F50" s="0">
+        <v>1312.5</v>
+      </c>
+      <c r="G50" s="0">
+        <v>4992.5</v>
+      </c>
+      <c r="H50" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x667744</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0">
+        <v>49</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Blue Cave #5</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blue Cave</t>
+        </is>
+      </c>
+      <c r="D51" s="0">
+        <v>26</v>
+      </c>
+      <c r="E51" s="0">
+        <v>5</v>
+      </c>
+      <c r="F51" s="0">
+        <v>2090</v>
+      </c>
+      <c r="G51" s="0">
+        <v>5192.5</v>
+      </c>
+      <c r="H51" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x667750</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0">
+        <v>50</v>
+      </c>
+      <c r="B52" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Blue Cave #6</t>
+        </is>
+      </c>
+      <c r="C52" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blue Cave</t>
+        </is>
+      </c>
+      <c r="D52" s="0">
+        <v>26</v>
+      </c>
+      <c r="E52" s="0">
+        <v>6</v>
+      </c>
+      <c r="F52" s="0">
+        <v>1797.5</v>
+      </c>
+      <c r="G52" s="0">
+        <v>5685</v>
+      </c>
+      <c r="H52" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x66775C</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="0">
+        <v>51</v>
+      </c>
+      <c r="B53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Blue Cave #7</t>
+        </is>
+      </c>
+      <c r="C53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blue Cave</t>
+        </is>
+      </c>
+      <c r="D53" s="0">
+        <v>26</v>
+      </c>
+      <c r="E53" s="0">
+        <v>7</v>
+      </c>
+      <c r="F53" s="0">
+        <v>-13.5</v>
+      </c>
+      <c r="G53" s="0">
+        <v>179.5</v>
+      </c>
+      <c r="H53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x667770</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="0">
+        <v>52</v>
+      </c>
+      <c r="B54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Cull Hazard #1</t>
+        </is>
+      </c>
+      <c r="C54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cull Hazard</t>
+        </is>
+      </c>
+      <c r="D54" s="0">
+        <v>27</v>
+      </c>
+      <c r="E54" s="0">
+        <v>1</v>
+      </c>
+      <c r="F54" s="0">
+        <v>1085</v>
+      </c>
+      <c r="G54" s="0">
+        <v>1320</v>
+      </c>
+      <c r="H54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x6C69D0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0">
+        <v>53</v>
+      </c>
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Cull Hazard #2</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cull Hazard</t>
+        </is>
+      </c>
+      <c r="D55" s="0">
+        <v>27</v>
+      </c>
+      <c r="E55" s="0">
+        <v>2</v>
+      </c>
+      <c r="F55" s="0">
+        <v>1422.5</v>
+      </c>
+      <c r="G55" s="0">
+        <v>1260</v>
+      </c>
+      <c r="H55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x6C69DC</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0">
+        <v>54</v>
+      </c>
+      <c r="B56" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Baragoon Tunnel (Shilf) #1</t>
+        </is>
+      </c>
+      <c r="C56" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baragoon Tunnel (Shilf)</t>
+        </is>
+      </c>
+      <c r="D56" s="0">
+        <v>28</v>
+      </c>
+      <c r="E56" s="0">
+        <v>1</v>
+      </c>
+      <c r="F56" s="0">
+        <v>-2880</v>
+      </c>
+      <c r="G56" s="0">
+        <v>-335</v>
+      </c>
+      <c r="H56" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x720D20</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="0">
+        <v>55</v>
+      </c>
+      <c r="B57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Baragoon Tunnel (Shilf) #2</t>
+        </is>
+      </c>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baragoon Tunnel (Shilf)</t>
+        </is>
+      </c>
+      <c r="D57" s="0">
+        <v>28</v>
+      </c>
+      <c r="E57" s="0">
+        <v>2</v>
+      </c>
+      <c r="F57" s="0">
+        <v>4725</v>
+      </c>
+      <c r="G57" s="0">
+        <v>1800</v>
+      </c>
+      <c r="H57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x720D2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0">
+        <v>56</v>
+      </c>
+      <c r="B58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Baragoon Tunnel (Shilf) #3</t>
+        </is>
+      </c>
+      <c r="C58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baragoon Tunnel (Shilf)</t>
+        </is>
+      </c>
+      <c r="D58" s="0">
+        <v>28</v>
+      </c>
+      <c r="E58" s="0">
+        <v>3</v>
+      </c>
+      <c r="F58" s="0">
+        <v>3012.5</v>
+      </c>
+      <c r="G58" s="0">
+        <v>1620</v>
+      </c>
+      <c r="H58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x720D38</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="0">
+        <v>57</v>
+      </c>
+      <c r="B59" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Baragoon Tunnel (Shilf) #4</t>
+        </is>
+      </c>
+      <c r="C59" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baragoon Tunnel (Shilf)</t>
+        </is>
+      </c>
+      <c r="D59" s="0">
+        <v>28</v>
+      </c>
+      <c r="E59" s="0">
+        <v>4</v>
+      </c>
+      <c r="F59" s="0">
+        <v>2847</v>
+      </c>
+      <c r="G59" s="0">
+        <v>1960</v>
+      </c>
+      <c r="H59" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x720D44</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="0">
+        <v>58</v>
+      </c>
+      <c r="B60" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Baragoon Tunnel (Shilf) #5</t>
+        </is>
+      </c>
+      <c r="C60" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baragoon Tunnel (Shilf)</t>
+        </is>
+      </c>
+      <c r="D60" s="0">
+        <v>28</v>
+      </c>
+      <c r="E60" s="0">
+        <v>5</v>
+      </c>
+      <c r="F60" s="0">
+        <v>-197.5</v>
+      </c>
+      <c r="G60" s="0">
+        <v>972.5</v>
+      </c>
+      <c r="H60" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x720D50</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="0">
+        <v>59</v>
+      </c>
+      <c r="B61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Boil Hole (Fargo) #1</t>
+        </is>
+      </c>
+      <c r="C61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Boil Hole (Fargo)</t>
+        </is>
+      </c>
+      <c r="D61" s="0">
+        <v>29</v>
+      </c>
+      <c r="E61" s="0">
+        <v>1</v>
+      </c>
+      <c r="F61" s="0">
+        <v>7174</v>
+      </c>
+      <c r="G61" s="0">
+        <v>-1274</v>
+      </c>
+      <c r="H61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x744A50</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="0">
+        <v>60</v>
+      </c>
+      <c r="B62" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Boil Hole (Fargo) #2</t>
+        </is>
+      </c>
+      <c r="C62" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Boil Hole (Fargo)</t>
+        </is>
+      </c>
+      <c r="D62" s="0">
+        <v>29</v>
+      </c>
+      <c r="E62" s="0">
+        <v>2</v>
+      </c>
+      <c r="F62" s="0">
+        <v>5272</v>
+      </c>
+      <c r="G62" s="0">
+        <v>1038</v>
+      </c>
+      <c r="H62" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x744A5C</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="0">
+        <v>61</v>
+      </c>
+      <c r="B63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Brannoch Castle #1</t>
+        </is>
+      </c>
+      <c r="C63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brannoch Castle</t>
+        </is>
+      </c>
+      <c r="D63" s="0">
+        <v>30</v>
+      </c>
+      <c r="E63" s="0">
+        <v>1</v>
+      </c>
+      <c r="F63" s="0">
+        <v>100</v>
+      </c>
+      <c r="G63" s="0">
+        <v>-100</v>
+      </c>
+      <c r="H63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x787880</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0">
+        <v>62</v>
+      </c>
+      <c r="B64" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Brannoch Castle #2</t>
+        </is>
+      </c>
+      <c r="C64" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brannoch Castle</t>
+        </is>
+      </c>
+      <c r="D64" s="0">
+        <v>30</v>
+      </c>
+      <c r="E64" s="0">
+        <v>2</v>
+      </c>
+      <c r="F64" s="0">
+        <v>76.5</v>
+      </c>
+      <c r="G64" s="0">
+        <v>-43.5</v>
+      </c>
+      <c r="H64" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x787890</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="0">
+        <v>63</v>
+      </c>
+      <c r="B65" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Connor Forest (Solvaring) #1</t>
+        </is>
+      </c>
+      <c r="C65" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Connor Forest (Solvaring)</t>
+        </is>
+      </c>
+      <c r="D65" s="0">
+        <v>31</v>
+      </c>
+      <c r="E65" s="0">
+        <v>1</v>
+      </c>
+      <c r="F65" s="0">
+        <v>-142</v>
+      </c>
+      <c r="G65" s="0">
+        <v>304</v>
+      </c>
+      <c r="H65" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x7C3EB0</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="0">
+        <v>64</v>
+      </c>
+      <c r="B66" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Connor Forest (Solvaring) #2</t>
+        </is>
+      </c>
+      <c r="C66" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Connor Forest (Solvaring)</t>
+        </is>
+      </c>
+      <c r="D66" s="0">
+        <v>31</v>
+      </c>
+      <c r="E66" s="0">
+        <v>2</v>
+      </c>
+      <c r="F66" s="0">
+        <v>1374</v>
+      </c>
+      <c r="G66" s="0">
+        <v>-940</v>
+      </c>
+      <c r="H66" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x7C3EBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0">
+        <v>65</v>
+      </c>
+      <c r="B67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Connor Forest (Solvaring) #3</t>
+        </is>
+      </c>
+      <c r="C67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Connor Forest (Solvaring)</t>
+        </is>
+      </c>
+      <c r="D67" s="0">
+        <v>31</v>
+      </c>
+      <c r="E67" s="0">
+        <v>3</v>
+      </c>
+      <c r="F67" s="0">
+        <v>2030</v>
+      </c>
+      <c r="G67" s="0">
+        <v>-142</v>
+      </c>
+      <c r="H67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x7C3EC8</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="0">
+        <v>66</v>
+      </c>
+      <c r="B68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Connor Forest (Solvaring) #4</t>
+        </is>
+      </c>
+      <c r="C68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Connor Forest (Solvaring)</t>
+        </is>
+      </c>
+      <c r="D68" s="0">
+        <v>31</v>
+      </c>
+      <c r="E68" s="0">
+        <v>4</v>
+      </c>
+      <c r="F68" s="0">
+        <v>-582</v>
+      </c>
+      <c r="G68" s="0">
+        <v>310</v>
+      </c>
+      <c r="H68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x7C3ED4</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0">
+        <v>67</v>
+      </c>
+      <c r="B69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Connor Forest (Solvaring) #5</t>
+        </is>
+      </c>
+      <c r="C69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Connor Forest (Solvaring)</t>
+        </is>
+      </c>
+      <c r="D69" s="0">
+        <v>31</v>
+      </c>
+      <c r="E69" s="0">
+        <v>5</v>
+      </c>
+      <c r="F69" s="0">
+        <v>5.15000009536743</v>
+      </c>
+      <c r="G69" s="0">
+        <v>2.84999990463257</v>
+      </c>
+      <c r="H69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x7C3EE0</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0">
+        <v>68</v>
+      </c>
+      <c r="B70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Glencoe Forest #1</t>
+        </is>
+      </c>
+      <c r="C70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Glencoe Forest</t>
+        </is>
+      </c>
+      <c r="D70" s="0">
+        <v>32</v>
+      </c>
+      <c r="E70" s="0">
+        <v>1</v>
+      </c>
+      <c r="F70" s="0">
+        <v>452</v>
+      </c>
+      <c r="G70" s="0">
+        <v>439</v>
+      </c>
+      <c r="H70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x7F1AB0</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0">
+        <v>69</v>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Glencoe Forest #2</t>
+        </is>
+      </c>
+      <c r="C71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Glencoe Forest</t>
+        </is>
+      </c>
+      <c r="D71" s="0">
+        <v>32</v>
+      </c>
+      <c r="E71" s="0">
+        <v>2</v>
+      </c>
+      <c r="F71" s="0">
+        <v>-298</v>
+      </c>
+      <c r="G71" s="0">
+        <v>333</v>
+      </c>
+      <c r="H71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x7F1ABC</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0">
+        <v>70</v>
+      </c>
+      <c r="B72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Glencoe Forest #3</t>
+        </is>
+      </c>
+      <c r="C72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Glencoe Forest</t>
+        </is>
+      </c>
+      <c r="D72" s="0">
+        <v>32</v>
+      </c>
+      <c r="E72" s="0">
+        <v>3</v>
+      </c>
+      <c r="F72" s="0">
+        <v>-721</v>
+      </c>
+      <c r="G72" s="0">
+        <v>326</v>
+      </c>
+      <c r="H72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x7F1AC8</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0">
+        <v>71</v>
+      </c>
+      <c r="B73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Glencoe Forest #4</t>
+        </is>
+      </c>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Glencoe Forest</t>
+        </is>
+      </c>
+      <c r="D73" s="0">
+        <v>32</v>
+      </c>
+      <c r="E73" s="0">
+        <v>4</v>
+      </c>
+      <c r="F73" s="0">
+        <v>-873</v>
+      </c>
+      <c r="G73" s="0">
+        <v>-722</v>
+      </c>
+      <c r="H73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x7F1AD4</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0">
+        <v>72</v>
+      </c>
+      <c r="B74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Glencoe Forest #5</t>
+        </is>
+      </c>
+      <c r="C74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Glencoe Forest</t>
+        </is>
+      </c>
+      <c r="D74" s="0">
+        <v>32</v>
+      </c>
+      <c r="E74" s="0">
+        <v>5</v>
+      </c>
+      <c r="F74" s="0">
+        <v>-1077</v>
+      </c>
+      <c r="G74" s="0">
+        <v>141</v>
+      </c>
+      <c r="H74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x7F1AE0</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0">
+        <v>73</v>
+      </c>
+      <c r="B75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Glencoe Forest #6</t>
+        </is>
+      </c>
+      <c r="C75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Glencoe Forest</t>
+        </is>
+      </c>
+      <c r="D75" s="0">
+        <v>32</v>
+      </c>
+      <c r="E75" s="0">
+        <v>6</v>
+      </c>
+      <c r="F75" s="0">
+        <v>-1330</v>
+      </c>
+      <c r="G75" s="0">
+        <v>177</v>
+      </c>
+      <c r="H75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x7F1AEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0">
+        <v>74</v>
+      </c>
+      <c r="B76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Windward Forest (Zelse) #1</t>
+        </is>
+      </c>
+      <c r="C76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Windward Forest (Zelse)</t>
+        </is>
+      </c>
+      <c r="D76" s="0">
+        <v>33</v>
+      </c>
+      <c r="E76" s="0">
+        <v>1</v>
+      </c>
+      <c r="F76" s="0">
+        <v>301</v>
+      </c>
+      <c r="G76" s="0">
+        <v>-159</v>
+      </c>
+      <c r="H76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x8253C0</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0">
+        <v>75</v>
+      </c>
+      <c r="B77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Windward Forest (Zelse) #2</t>
+        </is>
+      </c>
+      <c r="C77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Windward Forest (Zelse)</t>
+        </is>
+      </c>
+      <c r="D77" s="0">
+        <v>33</v>
+      </c>
+      <c r="E77" s="0">
+        <v>2</v>
+      </c>
+      <c r="F77" s="0">
+        <v>-494</v>
+      </c>
+      <c r="G77" s="0">
+        <v>189</v>
+      </c>
+      <c r="H77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x8253CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="0">
+        <v>76</v>
+      </c>
+      <c r="B78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Windward Forest (Zelse) #3</t>
+        </is>
+      </c>
+      <c r="C78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Windward Forest (Zelse)</t>
+        </is>
+      </c>
+      <c r="D78" s="0">
+        <v>33</v>
+      </c>
+      <c r="E78" s="0">
+        <v>3</v>
+      </c>
+      <c r="F78" s="0">
+        <v>450</v>
+      </c>
+      <c r="G78" s="0">
+        <v>225</v>
+      </c>
+      <c r="H78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x8253D8</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="0">
+        <v>77</v>
+      </c>
+      <c r="B79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Windward Forest (Zelse) #4</t>
+        </is>
+      </c>
+      <c r="C79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Windward Forest (Zelse)</t>
+        </is>
+      </c>
+      <c r="D79" s="0">
+        <v>33</v>
+      </c>
+      <c r="E79" s="0">
+        <v>4</v>
+      </c>
+      <c r="F79" s="0">
+        <v>-4</v>
+      </c>
+      <c r="G79" s="0">
+        <v>25</v>
+      </c>
+      <c r="H79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x8253F0</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="0">
+        <v>78</v>
+      </c>
+      <c r="B80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dondoran Castle #1</t>
+        </is>
+      </c>
+      <c r="C80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dondoran Castle</t>
+        </is>
+      </c>
+      <c r="D80" s="0">
+        <v>14</v>
+      </c>
+      <c r="E80" s="0">
+        <v>1</v>
+      </c>
+      <c r="F80" s="0">
+        <v>16</v>
+      </c>
+      <c r="G80" s="0">
+        <v>0</v>
+      </c>
+      <c r="H80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x489840</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="0">
+        <v>79</v>
+      </c>
+      <c r="B81" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dondoran Castle #2</t>
+        </is>
+      </c>
+      <c r="C81" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dondoran Castle</t>
+        </is>
+      </c>
+      <c r="D81" s="0">
+        <v>14</v>
+      </c>
+      <c r="E81" s="0">
+        <v>2</v>
+      </c>
+      <c r="F81" s="0">
+        <v>-22.5</v>
+      </c>
+      <c r="G81" s="0">
+        <v>31.5</v>
+      </c>
+      <c r="H81" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x489850</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="0">
+        <v>80</v>
+      </c>
+      <c r="B82" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dondoran buildings #1</t>
+        </is>
+      </c>
+      <c r="C82" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dondoran buildings</t>
+        </is>
+      </c>
+      <c r="D82" s="0">
+        <v>16</v>
+      </c>
+      <c r="E82" s="0">
+        <v>1</v>
+      </c>
+      <c r="F82" s="0">
+        <v>-22</v>
+      </c>
+      <c r="G82" s="0">
+        <v>-19</v>
+      </c>
+      <c r="H82" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x4CF140</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="0">
+        <v>81</v>
+      </c>
+      <c r="B83" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Limelin Castle #1</t>
+        </is>
+      </c>
+      <c r="C83" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limelin Castle</t>
+        </is>
+      </c>
+      <c r="D83" s="0">
+        <v>21</v>
+      </c>
+      <c r="E83" s="0">
+        <v>1</v>
+      </c>
+      <c r="F83" s="0">
+        <v>-5</v>
+      </c>
+      <c r="G83" s="0">
+        <v>80</v>
+      </c>
+      <c r="H83" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x56FAC0</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="0">
+        <v>82</v>
+      </c>
+      <c r="B84" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Limelin Castle #2</t>
+        </is>
+      </c>
+      <c r="C84" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limelin Castle</t>
+        </is>
+      </c>
+      <c r="D84" s="0">
+        <v>21</v>
+      </c>
+      <c r="E84" s="0">
+        <v>2</v>
+      </c>
+      <c r="F84" s="0">
+        <v>5</v>
+      </c>
+      <c r="G84" s="0">
+        <v>80</v>
+      </c>
+      <c r="H84" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x56FACC</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="0">
+        <v>83</v>
+      </c>
+      <c r="B85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Limelin Castle #3</t>
+        </is>
+      </c>
+      <c r="C85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limelin Castle</t>
+        </is>
+      </c>
+      <c r="D85" s="0">
+        <v>21</v>
+      </c>
+      <c r="E85" s="0">
+        <v>3</v>
+      </c>
+      <c r="F85" s="0">
+        <v>-53</v>
+      </c>
+      <c r="G85" s="0">
+        <v>28</v>
+      </c>
+      <c r="H85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x56FAE0</t>
+        </is>
+      </c>
+      <c r="I85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hidden inside the return ship (Limelin to Dondoran); "Reveal hidden spirits" moves it out</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="0">
+        <v>84</v>
+      </c>
+      <c r="B86" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Limelin buildings #1</t>
+        </is>
+      </c>
+      <c r="C86" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limelin buildings</t>
+        </is>
+      </c>
+      <c r="D86" s="0">
+        <v>22</v>
+      </c>
+      <c r="E86" s="0">
+        <v>1</v>
+      </c>
+      <c r="F86" s="0">
+        <v>0</v>
+      </c>
+      <c r="G86" s="0">
+        <v>0</v>
+      </c>
+      <c r="H86" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x59F590</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="0">
+        <v>85</v>
+      </c>
+      <c r="B87" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Limelin buildings #2</t>
+        </is>
+      </c>
+      <c r="C87" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limelin buildings</t>
+        </is>
+      </c>
+      <c r="D87" s="0">
+        <v>22</v>
+      </c>
+      <c r="E87" s="0">
+        <v>2</v>
+      </c>
+      <c r="F87" s="0">
+        <v>-5</v>
+      </c>
+      <c r="G87" s="0">
+        <v>25</v>
+      </c>
+      <c r="H87" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x59F5A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="0">
+        <v>86</v>
+      </c>
+      <c r="B88" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Limelin buildings #3</t>
+        </is>
+      </c>
+      <c r="C88" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limelin buildings</t>
+        </is>
+      </c>
+      <c r="D88" s="0">
+        <v>22</v>
+      </c>
+      <c r="E88" s="0">
+        <v>3</v>
+      </c>
+      <c r="F88" s="0">
+        <v>-32</v>
+      </c>
+      <c r="G88" s="0">
+        <v>-20.5</v>
+      </c>
+      <c r="H88" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x59F5AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="0">
+        <v>87</v>
+      </c>
+      <c r="B89" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dindom Dries &amp; Brannoch buildings #1</t>
+        </is>
+      </c>
+      <c r="C89" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dindom Dries &amp; Brannoch buildings</t>
+        </is>
+      </c>
+      <c r="D89" s="0">
+        <v>23</v>
+      </c>
+      <c r="E89" s="0">
+        <v>1</v>
+      </c>
+      <c r="F89" s="0">
+        <v>27</v>
+      </c>
+      <c r="G89" s="0">
+        <v>27.5</v>
+      </c>
+      <c r="H89" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x5D8AF0</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="0">
+        <v>88</v>
+      </c>
+      <c r="B90" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Dindom Dries &amp; Brannoch buildings #2</t>
+        </is>
+      </c>
+      <c r="C90" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dindom Dries &amp; Brannoch buildings</t>
+        </is>
+      </c>
+      <c r="D90" s="0">
+        <v>23</v>
+      </c>
+      <c r="E90" s="0">
+        <v>2</v>
+      </c>
+      <c r="F90" s="0">
+        <v>4.5</v>
+      </c>
+      <c r="G90" s="0">
+        <v>5.5</v>
+      </c>
+      <c r="H90" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x5D8B00</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="0">
+        <v>89</v>
+      </c>
+      <c r="B91" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Shamwood buildings #1</t>
+        </is>
+      </c>
+      <c r="C91" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shamwood buildings</t>
+        </is>
+      </c>
+      <c r="D91" s="0">
+        <v>24</v>
+      </c>
+      <c r="E91" s="0">
+        <v>1</v>
+      </c>
+      <c r="F91" s="0">
+        <v>-25</v>
+      </c>
+      <c r="G91" s="0">
+        <v>25</v>
+      </c>
+      <c r="H91" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x5EBAC0</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="0">
+        <v>90</v>
+      </c>
+      <c r="B92" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Shamwood buildings #2</t>
+        </is>
+      </c>
+      <c r="C92" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shamwood buildings</t>
+        </is>
+      </c>
+      <c r="D92" s="0">
+        <v>24</v>
+      </c>
+      <c r="E92" s="0">
+        <v>2</v>
+      </c>
+      <c r="F92" s="0">
+        <v>25</v>
+      </c>
+      <c r="G92" s="0">
+        <v>25</v>
+      </c>
+      <c r="H92" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x5EBACC</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="0">
+        <v>91</v>
+      </c>
+      <c r="B93" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Shamwood buildings #3</t>
+        </is>
+      </c>
+      <c r="C93" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shamwood buildings</t>
+        </is>
+      </c>
+      <c r="D93" s="0">
+        <v>24</v>
+      </c>
+      <c r="E93" s="0">
+        <v>3</v>
+      </c>
+      <c r="F93" s="0">
+        <v>-25</v>
+      </c>
+      <c r="G93" s="0">
+        <v>-25</v>
+      </c>
+      <c r="H93" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x5EBAD8</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="0">
+        <v>92</v>
+      </c>
+      <c r="B94" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Shamwood buildings #4</t>
+        </is>
+      </c>
+      <c r="C94" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shamwood buildings</t>
+        </is>
+      </c>
+      <c r="D94" s="0">
+        <v>24</v>
+      </c>
+      <c r="E94" s="0">
+        <v>4</v>
+      </c>
+      <c r="F94" s="0">
+        <v>25</v>
+      </c>
+      <c r="G94" s="0">
+        <v>-25</v>
+      </c>
+      <c r="H94" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x5EBAE4</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="0">
+        <v>93</v>
+      </c>
+      <c r="B95" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Shamwood buildings #5</t>
+        </is>
+      </c>
+      <c r="C95" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shamwood buildings</t>
+        </is>
+      </c>
+      <c r="D95" s="0">
+        <v>24</v>
+      </c>
+      <c r="E95" s="0">
+        <v>5</v>
+      </c>
+      <c r="F95" s="0">
+        <v>10</v>
+      </c>
+      <c r="G95" s="0">
+        <v>80</v>
+      </c>
+      <c r="H95" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x5EBAF0</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="0">
+        <v>94</v>
+      </c>
+      <c r="B96" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Shamwood buildings #6</t>
+        </is>
+      </c>
+      <c r="C96" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shamwood buildings</t>
+        </is>
+      </c>
+      <c r="D96" s="0">
+        <v>24</v>
+      </c>
+      <c r="E96" s="0">
+        <v>6</v>
+      </c>
+      <c r="F96" s="0">
+        <v>-10</v>
+      </c>
+      <c r="G96" s="0">
+        <v>80</v>
+      </c>
+      <c r="H96" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x5EBAFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="0">
+        <v>95</v>
+      </c>
+      <c r="B97" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Hidden rooms &amp; shrines #1</t>
+        </is>
+      </c>
+      <c r="C97" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hidden rooms &amp; shrines</t>
+        </is>
+      </c>
+      <c r="D97" s="0">
+        <v>25</v>
+      </c>
+      <c r="E97" s="0">
+        <v>1</v>
+      </c>
+      <c r="F97" s="0">
+        <v>27</v>
+      </c>
+      <c r="G97" s="0">
+        <v>13.5</v>
+      </c>
+      <c r="H97" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x609950</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="0">
+        <v>96</v>
+      </c>
+      <c r="B98" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Hidden rooms &amp; shrines #2</t>
+        </is>
+      </c>
+      <c r="C98" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hidden rooms &amp; shrines</t>
+        </is>
+      </c>
+      <c r="D98" s="0">
+        <v>25</v>
+      </c>
+      <c r="E98" s="0">
+        <v>2</v>
+      </c>
+      <c r="F98" s="0">
+        <v>18</v>
+      </c>
+      <c r="G98" s="0">
+        <v>-7</v>
+      </c>
+      <c r="H98" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x609960</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="0">
+        <v>97</v>
+      </c>
+      <c r="B99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spirit - Hidden rooms &amp; shrines #3</t>
+        </is>
+      </c>
+      <c r="C99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hidden rooms &amp; shrines</t>
+        </is>
+      </c>
+      <c r="D99" s="0">
+        <v>25</v>
+      </c>
+      <c r="E99" s="0">
+        <v>3</v>
+      </c>
+      <c r="F99" s="0">
+        <v>-34</v>
+      </c>
+      <c r="G99" s="0">
+        <v>25</v>
+      </c>
+      <c r="H99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0x609970</t>
+        </is>
+      </c>
+      <c r="I99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hidden inside the Limelin Castle library; "Reveal hidden spirits" moves it out</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I99"/>
+</worksheet>
 </file>
</xml_diff>